<commit_message>
Final Board Order Changes
</commit_message>
<xml_diff>
--- a/DemoBoard/inspireFly_PQ_payloadDemo_rev0.1.xlsx
+++ b/DemoBoard/inspireFly_PQ_payloadDemo_rev0.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shane\Documents\GitHub\Pocketqube-Payload-Boards\DemoBoard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EF7B1B0-98B7-45B3-8F57-10224994860E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E60E50C-15B1-4EA8-83A1-1B9E9FD4DE5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="12870" windowHeight="12863" xr2:uid="{90A7F372-49DC-4743-8A39-617F3F98A630}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{90A7F372-49DC-4743-8A39-617F3F98A630}"/>
   </bookViews>
   <sheets>
     <sheet name="Ordering Sheet" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="128">
   <si>
     <t>Part Number</t>
   </si>
@@ -373,12 +373,6 @@
     <t>RES SMD 5.1K OHM 0.1% 1/16W 0402</t>
   </si>
   <si>
-    <t>RC0402FR-0727R4L</t>
-  </si>
-  <si>
-    <t>RES 27.4 OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
     <t>SC0914(13)</t>
   </si>
   <si>
@@ -410,6 +404,24 @@
   </si>
   <si>
     <t>CONN MICROSD CARD R/A SMD</t>
+  </si>
+  <si>
+    <t>RP73PF1E27R4BTD</t>
+  </si>
+  <si>
+    <t>RES 27.4 OHM 0.1% 1/10W 0402</t>
+  </si>
+  <si>
+    <t>LTST-C190KSKT</t>
+  </si>
+  <si>
+    <t>LTST-S270KRKT</t>
+  </si>
+  <si>
+    <t>LED RED CLEAR CHIP SMD R/A</t>
+  </si>
+  <si>
+    <t>LED YELLOW CLEAR CHIP SMD</t>
   </si>
 </sst>
 </file>
@@ -797,7 +809,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5925212D-D2B1-4AA1-8E95-17EB777828EB}">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.6640625" customWidth="1"/>
@@ -878,7 +890,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="G3" s="2">
-        <f t="shared" ref="G3:G25" si="0" xml:space="preserve"> E3 *F3</f>
+        <f t="shared" ref="G3:G26" si="0" xml:space="preserve"> E3 *F3</f>
         <v>0.12</v>
       </c>
     </row>
@@ -1037,10 +1049,10 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="D10">
         <v>2</v>
@@ -1050,11 +1062,11 @@
         <v>10</v>
       </c>
       <c r="F10" s="4">
-        <v>7.0000000000000001E-3</v>
+        <v>0.18</v>
       </c>
       <c r="G10" s="2">
         <f t="shared" si="0"/>
-        <v>7.0000000000000007E-2</v>
+        <v>1.7999999999999998</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
@@ -1068,18 +1080,18 @@
         <v>20</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11">
         <f xml:space="preserve"> D11 *Constants!$C$1</f>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F11" s="4">
         <v>8.2000000000000003E-2</v>
       </c>
       <c r="G11" s="2">
         <f t="shared" si="0"/>
-        <v>0.41000000000000003</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
@@ -1112,24 +1124,24 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C13" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13">
         <f xml:space="preserve"> D13 *Constants!$C$1</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F13" s="4">
         <v>0.7</v>
       </c>
       <c r="G13" s="2">
         <f t="shared" si="0"/>
-        <v>3.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
@@ -1137,10 +1149,10 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C14" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1162,10 +1174,10 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C15" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1215,7 +1227,7 @@
         <v>82</v>
       </c>
       <c r="C17" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -1240,7 +1252,7 @@
         <v>84</v>
       </c>
       <c r="C18" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1265,7 +1277,7 @@
         <v>87</v>
       </c>
       <c r="C19" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1365,7 +1377,7 @@
         <v>97</v>
       </c>
       <c r="C23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1390,7 +1402,7 @@
         <v>100</v>
       </c>
       <c r="C24" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -1411,6 +1423,12 @@
       <c r="A25" t="s">
         <v>10</v>
       </c>
+      <c r="B25" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C25" t="s">
+        <v>127</v>
+      </c>
       <c r="D25">
         <v>1</v>
       </c>
@@ -1418,18 +1436,46 @@
         <f xml:space="preserve"> D25 *Constants!$C$1</f>
         <v>5</v>
       </c>
+      <c r="F25" s="4">
+        <v>0.12</v>
+      </c>
       <c r="G25" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" ref="G25" si="1" xml:space="preserve"> E25 *F25</f>
+        <v>0.6</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C26" t="s">
+        <v>126</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <f xml:space="preserve"> D26 *Constants!$C$1</f>
+        <v>5</v>
+      </c>
+      <c r="F26" s="4">
+        <v>0.12</v>
+      </c>
+      <c r="G26" s="2">
+        <f t="shared" si="0"/>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
         <v>33</v>
       </c>
-      <c r="G26" s="2">
-        <f>SUM(G2:G25)</f>
-        <v>74.83499999999998</v>
+      <c r="G27" s="2">
+        <f>SUM(G2:G26)</f>
+        <v>82.084999999999994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>